<commit_message>
Regenerate Excel with priority-ordered actions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mi2nCubX9CDNDXvSBmxN1B
</commit_message>
<xml_diff>
--- a/stemon-competitor-analysis/STEAM教育_競合比較_元データ.xlsx
+++ b/stemon-competitor-analysis/STEAM教育_競合比較_元データ.xlsx
@@ -13824,6 +13824,12 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">成果の見える化</t>
+  </si>
+  <si>
+    <t xml:space="preserve">作品持ち帰り＋毎回の保護者レポート（写真・コメント）を標準化し、ロボ団・プログラボとの差別化軸にする</t>
+  </si>
+  <si>
     <t xml:space="preserve">カリキュラム</t>
   </si>
   <si>
@@ -13996,12 +14002,6 @@
       </rPr>
       <t xml:space="preserve">か月</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">成果の見える化</t>
-  </si>
-  <si>
-    <t xml:space="preserve">作品持ち帰り＋毎回の保護者レポート（写真・コメント）を標準化し、ロボ団・プログラボとの差別化軸にする</t>
   </si>
   <si>
     <t xml:space="preserve">集客・ターゲット</t>
@@ -16611,11 +16611,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="17110961"/>
-        <c:axId val="78971122"/>
+        <c:axId val="4973825"/>
+        <c:axId val="13356539"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="17110961"/>
+        <c:axId val="4973825"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -16647,7 +16647,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78971122"/>
+        <c:crossAx val="13356539"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -16655,7 +16655,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="78971122"/>
+        <c:axId val="13356539"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -16687,7 +16687,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17110961"/>
+        <c:crossAx val="4973825"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -21328,36 +21328,36 @@
       <c r="C21" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="D21" s="39" t="s">
-        <v>507</v>
+      <c r="D21" s="33" t="s">
+        <v>504</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="38" t="s">
+        <v>507</v>
+      </c>
+      <c r="B22" s="15" t="s">
         <v>508</v>
       </c>
-      <c r="B22" s="15" t="s">
+      <c r="C22" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="D22" s="39" t="s">
         <v>509</v>
-      </c>
-      <c r="C22" s="33" t="s">
-        <v>57</v>
-      </c>
-      <c r="D22" s="33" t="s">
-        <v>510</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="38" t="s">
+        <v>510</v>
+      </c>
+      <c r="B23" s="15" t="s">
         <v>511</v>
       </c>
-      <c r="B23" s="15" t="s">
+      <c r="C23" s="33" t="s">
+        <v>57</v>
+      </c>
+      <c r="D23" s="33" t="s">
         <v>512</v>
-      </c>
-      <c r="C23" s="33" t="s">
-        <v>68</v>
-      </c>
-      <c r="D23" s="33" t="s">
-        <v>504</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21385,7 +21385,7 @@
         <v>57</v>
       </c>
       <c r="D25" s="39" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>